<commit_message>
playing around with eleventy and python
</commit_message>
<xml_diff>
--- a/xlsx/ReplaceIVTFFtoTEI.xlsx
+++ b/xlsx/ReplaceIVTFFtoTEI.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hadle\Documents\GitHub\voynichTEI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hadle\Documents\GitHub\voynichTEI\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B60D8347-5E46-4719-B933-22226193E32B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E91E7501-87FE-4E52-92B3-BAE819CF6AD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DF9BB7F7-DEE6-4231-B8AE-192266D5BB45}"/>
+    <workbookView xWindow="10800" yWindow="264" windowWidth="11664" windowHeight="11952" xr2:uid="{DF9BB7F7-DEE6-4231-B8AE-192266D5BB45}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="428">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="430">
   <si>
     <t>Voynich</t>
   </si>
@@ -1322,6 +1322,12 @@
   </si>
   <si>
     <t>&lt;/zone&gt;</t>
+  </si>
+  <si>
+    <t>&lt;f\d+[rv]\d?\.(\d+),([@+*=&amp;~/!])([PLCR][01bcrtafnpstxzio])&gt;\s+(.+)</t>
+  </si>
+  <si>
+    <t>&lt;line n="\1" rendition="#\2 #\3"&gt;\4&lt;/line&gt;</t>
   </si>
 </sst>
 </file>
@@ -1776,8 +1782,8 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="28.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="44.5546875" customWidth="1"/>
+    <col min="8" max="8" width="28.5546875" customWidth="1"/>
     <col min="10" max="10" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="49" customWidth="1"/>
   </cols>
@@ -1838,6 +1844,12 @@
       <c r="E3" s="4">
         <v>7.5</v>
       </c>
+      <c r="G3" t="s">
+        <v>428</v>
+      </c>
+      <c r="H3" t="s">
+        <v>429</v>
+      </c>
       <c r="J3" s="8" t="s">
         <v>172</v>
       </c>

</xml_diff>

<commit_message>
new ixml experiments w/ python
</commit_message>
<xml_diff>
--- a/xlsx/ReplaceIVTFFtoTEI.xlsx
+++ b/xlsx/ReplaceIVTFFtoTEI.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hadle\Documents\GitHub\voynichTEI\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E91E7501-87FE-4E52-92B3-BAE819CF6AD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64762BD3-5AFA-42F4-A7BE-920D02ADB5F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10800" yWindow="264" windowWidth="11664" windowHeight="11952" xr2:uid="{DF9BB7F7-DEE6-4231-B8AE-192266D5BB45}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029" iterate="1" iterateCount="500"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>